<commit_message>
fix: some repair in livewire based on scenario testing
</commit_message>
<xml_diff>
--- a/docs/testing/livewire-test-scenarios.xlsx
+++ b/docs/testing/livewire-test-scenarios.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowWidth="29400" windowHeight="13940" tabRatio="860" firstSheet="11" activeTab="11"/>
+    <workbookView windowWidth="29400" windowHeight="13140" tabRatio="860"/>
   </bookViews>
   <sheets>
     <sheet name="INDEX" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2018" uniqueCount="1222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2022" uniqueCount="1228">
   <si>
     <t>No</t>
   </si>
@@ -1851,6 +1851,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">Centang pokok (locked) </t>
     </r>
     <r>
@@ -2200,6 +2206,9 @@
     <t>Withdrawal status draft</t>
   </si>
   <si>
+    <t>ketika jenis pencairan transfer, tampilkan juga bank dan nomor rekening tujuan</t>
+  </si>
+  <si>
     <t>LW-WDR-03</t>
   </si>
   <si>
@@ -2326,6 +2335,9 @@
     <t>Kosongkan period_year → save</t>
   </si>
   <si>
+    <t xml:space="preserve">perhatikan ulang ini. ketika pindah tahun atau di luar periode, masih ada. harusnya tidak </t>
+  </si>
+  <si>
     <t>LW-WDR-12</t>
   </si>
   <si>
@@ -2476,6 +2488,9 @@
     <t>LW-SHP-09</t>
   </si>
   <si>
+    <t>aksinya sudah dibatasi tapi masih muncul button revresal</t>
+  </si>
+  <si>
     <t>LW-HOL-01</t>
   </si>
   <si>
@@ -2662,6 +2677,9 @@
     <t>User dibuat, password ter-hash, roles ter-sync</t>
   </si>
   <si>
+    <t>kalau bisa password tu generate otomatis</t>
+  </si>
+  <si>
     <t>LW-USR-02</t>
   </si>
   <si>
@@ -3043,6 +3061,9 @@
     <t>Isi semua rate/amount valid → save</t>
   </si>
   <si>
+    <t>belum implementasi yang rupiah</t>
+  </si>
+  <si>
     <t>LW-SET-08</t>
   </si>
   <si>
@@ -3344,6 +3365,9 @@
   </si>
   <si>
     <t>Notifikasi verifikasi dikirim</t>
+  </si>
+  <si>
+    <t>ketika loading kirim, tulisan jadi loading - menutup kemungkinan user bingung dan double click</t>
   </si>
   <si>
     <t>LW-PRF-07</t>
@@ -3957,7 +3981,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3973,6 +3997,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4314,7 +4344,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -4338,16 +4368,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -4356,89 +4386,89 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -4449,13 +4479,16 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4465,7 +4498,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" quotePrefix="1">
       <alignment vertical="top"/>
@@ -5509,7 +5547,7 @@
       <c r="D2" s="2" t="s">
         <v>588</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="6" t="s">
         <v>589</v>
       </c>
       <c r="F2" s="2" t="s">
@@ -5966,7 +6004,7 @@
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="I3" s="3"/>
     </row>
     <row r="4" ht="34" spans="1:9">
       <c r="A4" s="2" t="s">
@@ -5989,7 +6027,7 @@
       </c>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="I4" s="3"/>
     </row>
     <row r="5" ht="17" spans="1:9">
       <c r="A5" s="2" t="s">
@@ -6014,7 +6052,7 @@
         <v>487</v>
       </c>
       <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="I5" s="3"/>
     </row>
     <row r="6" ht="34" spans="1:9">
       <c r="A6" s="2" t="s">
@@ -6039,7 +6077,7 @@
         <v>487</v>
       </c>
       <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
+      <c r="I6" s="3"/>
     </row>
     <row r="7" ht="34" spans="1:9">
       <c r="A7" s="2" t="s">
@@ -6062,7 +6100,7 @@
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="I7" s="3"/>
     </row>
     <row r="8" ht="17" spans="1:9">
       <c r="A8" s="2" t="s">
@@ -6085,7 +6123,7 @@
       </c>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="I8" s="3"/>
     </row>
     <row r="9" ht="17" spans="1:9">
       <c r="A9" s="2" t="s">
@@ -6108,7 +6146,7 @@
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="I9" s="3"/>
     </row>
     <row r="10" ht="34" spans="1:9">
       <c r="A10" s="2" t="s">
@@ -6131,7 +6169,7 @@
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="I10" s="3"/>
     </row>
     <row r="11" ht="17" spans="1:9">
       <c r="A11" s="2" t="s">
@@ -6154,7 +6192,7 @@
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="I11" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6231,7 +6269,7 @@
         <v>487</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="3" ht="34" spans="1:9">
       <c r="A3" s="2" t="s">
@@ -6253,192 +6291,192 @@
         <v>698</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>487</v>
+        <v>699</v>
       </c>
       <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="I3" s="3"/>
     </row>
     <row r="4" ht="17" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="I4" s="3"/>
     </row>
     <row r="5" ht="34" spans="1:9">
       <c r="A5" s="2" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="I5" s="3"/>
     </row>
     <row r="6" ht="17" spans="1:9">
       <c r="A6" s="2" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
+      <c r="I6" s="3"/>
     </row>
     <row r="7" ht="34" spans="1:9">
       <c r="A7" s="2" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="I7" s="3"/>
     </row>
     <row r="8" ht="34" spans="1:9">
       <c r="A8" s="2" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="I8" s="3"/>
     </row>
     <row r="9" ht="17" spans="1:9">
       <c r="A9" s="2" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="I9" s="3"/>
     </row>
     <row r="10" ht="34" spans="1:9">
       <c r="A10" s="2" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="I10" s="3"/>
     </row>
     <row r="11" ht="17" spans="1:9">
       <c r="A11" s="2" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>80</v>
@@ -6447,7 +6485,7 @@
         <v>81</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>439</v>
@@ -6456,137 +6494,139 @@
         <v>487</v>
       </c>
       <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-    </row>
-    <row r="12" ht="17" spans="1:9">
+      <c r="I11" s="3"/>
+    </row>
+    <row r="12" ht="51" spans="1:9">
       <c r="A12" s="2" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="G12" s="2"/>
+      <c r="G12" s="2" t="s">
+        <v>742</v>
+      </c>
       <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="I12" s="5"/>
     </row>
     <row r="13" ht="17" spans="1:9">
       <c r="A13" s="2" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
+      <c r="I13" s="3"/>
     </row>
     <row r="14" ht="17" spans="1:9">
       <c r="A14" s="2" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="I14" s="3"/>
     </row>
     <row r="15" ht="17" spans="1:9">
       <c r="A15" s="2" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+      <c r="I15" s="3"/>
     </row>
     <row r="16" ht="17" spans="1:9">
       <c r="A16" s="2" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
+      <c r="I16" s="3"/>
     </row>
     <row r="17" ht="17" spans="1:9">
       <c r="A17" s="2" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>80</v>
@@ -6598,13 +6638,13 @@
         <v>510</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
+      <c r="I17" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6616,8 +6656,8 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="7"/>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -6626,9 +6666,10 @@
     <col min="5" max="5" width="34" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="33.0703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:8">
+    <row r="1" ht="22" customHeight="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>59</v>
       </c>
@@ -6654,78 +6695,78 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" ht="17" spans="1:8">
+    <row r="2" ht="17" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" ht="17" spans="1:8">
+      <c r="H2" s="3"/>
+    </row>
+    <row r="3" ht="17" spans="1:9">
       <c r="A3" s="2" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" ht="34" spans="1:8">
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" ht="34" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>515</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" ht="51" spans="1:8">
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" ht="51" spans="1:9">
       <c r="A5" s="2" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
@@ -6734,20 +6775,20 @@
         <v>81</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" ht="17" spans="1:8">
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" ht="17" spans="1:9">
       <c r="A6" s="2" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
@@ -6762,14 +6803,14 @@
         <v>161</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" ht="17" spans="1:8">
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" ht="17" spans="1:9">
       <c r="A7" s="2" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>80</v>
@@ -6778,20 +6819,20 @@
         <v>81</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" ht="17" spans="1:8">
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" ht="17" spans="1:9">
       <c r="A8" s="2" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>80</v>
@@ -6800,20 +6841,20 @@
         <v>81</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>414</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" ht="17" spans="1:8">
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" ht="17" spans="1:9">
       <c r="A9" s="2" t="s">
-        <v>788</v>
+        <v>790</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>80</v>
@@ -6828,11 +6869,11 @@
         <v>273</v>
       </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" ht="17" spans="1:8">
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" ht="17" spans="1:9">
       <c r="A10" s="2" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>652</v>
@@ -6850,7 +6891,10 @@
         <v>536</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="H10" s="4"/>
+      <c r="I10" t="s">
+        <v>793</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6902,54 +6946,54 @@
     </row>
     <row r="2" ht="34" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>791</v>
+        <v>794</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>792</v>
+        <v>795</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>793</v>
+        <v>796</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>794</v>
+        <v>797</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>795</v>
+        <v>798</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" ht="17" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>796</v>
+        <v>799</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>799</v>
+        <v>802</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>322</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" ht="17" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>800</v>
+        <v>803</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
@@ -6958,20 +7002,20 @@
         <v>81</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>802</v>
+        <v>805</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>803</v>
+        <v>806</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" ht="17" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>804</v>
+        <v>807</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>805</v>
+        <v>808</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
@@ -6983,39 +7027,39 @@
         <v>151</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>806</v>
+        <v>809</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" ht="17" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>807</v>
+        <v>810</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>808</v>
+        <v>811</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>809</v>
+        <v>812</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>510</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>810</v>
+        <v>813</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" ht="17" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>811</v>
+        <v>814</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>812</v>
+        <v>815</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>69</v>
@@ -7030,36 +7074,36 @@
         <v>161</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="H7" s="3"/>
     </row>
     <row r="8" ht="17" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>813</v>
+        <v>816</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>814</v>
+        <v>817</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>815</v>
+        <v>818</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>816</v>
+        <v>819</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>817</v>
+        <v>820</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="H8" s="3"/>
     </row>
     <row r="9" ht="17" spans="1:8">
       <c r="A9" s="2" t="s">
-        <v>818</v>
+        <v>821</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>819</v>
+        <v>822</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>80</v>
@@ -7068,20 +7112,20 @@
         <v>81</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>820</v>
+        <v>823</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>422</v>
       </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+      <c r="H9" s="3"/>
     </row>
     <row r="10" ht="17" spans="1:8">
       <c r="A10" s="2" t="s">
-        <v>821</v>
+        <v>824</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>822</v>
+        <v>825</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>80</v>
@@ -7090,13 +7134,13 @@
         <v>81</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>823</v>
+        <v>826</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>414</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="H10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7148,10 +7192,10 @@
     </row>
     <row r="2" ht="17" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>824</v>
+        <v>827</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>825</v>
+        <v>828</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
@@ -7160,20 +7204,20 @@
         <v>159</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>826</v>
+        <v>829</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>827</v>
+        <v>830</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" ht="17" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>828</v>
+        <v>831</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>829</v>
+        <v>832</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
@@ -7188,36 +7232,36 @@
         <v>161</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" ht="17" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>830</v>
+        <v>833</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>831</v>
+        <v>834</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>832</v>
+        <v>835</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>833</v>
+        <v>836</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>834</v>
+        <v>837</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" ht="17" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>835</v>
+        <v>838</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>836</v>
+        <v>839</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
@@ -7226,42 +7270,42 @@
         <v>81</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>837</v>
+        <v>840</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>838</v>
+        <v>841</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" ht="17" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>839</v>
+        <v>842</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>840</v>
+        <v>843</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>841</v>
+        <v>844</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>842</v>
+        <v>845</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>843</v>
+        <v>846</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" ht="17" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>844</v>
+        <v>847</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>845</v>
+        <v>848</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>80</v>
@@ -7270,13 +7314,13 @@
         <v>81</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>846</v>
+        <v>849</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>847</v>
+        <v>850</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="H7" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7332,35 +7376,35 @@
     </row>
     <row r="2" ht="17" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>848</v>
+        <v>851</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>849</v>
+        <v>852</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>850</v>
+        <v>853</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>851</v>
+        <v>854</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>852</v>
+        <v>855</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>487</v>
+        <v>856</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="3" ht="17" spans="1:9">
       <c r="A3" s="2" t="s">
-        <v>853</v>
+        <v>857</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>854</v>
+        <v>858</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
@@ -7369,23 +7413,23 @@
         <v>81</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>855</v>
+        <v>859</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>856</v>
+        <v>860</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="I3" s="3"/>
     </row>
     <row r="4" ht="17" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>857</v>
+        <v>861</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>858</v>
+        <v>862</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
@@ -7394,23 +7438,23 @@
         <v>86</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>859</v>
+        <v>863</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="I4" s="3"/>
     </row>
     <row r="5" ht="17" spans="1:9">
       <c r="A5" s="2" t="s">
-        <v>861</v>
+        <v>865</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>862</v>
+        <v>866</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
@@ -7428,14 +7472,14 @@
         <v>487</v>
       </c>
       <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="I5" s="3"/>
     </row>
     <row r="6" ht="17" spans="1:9">
       <c r="A6" s="2" t="s">
-        <v>863</v>
+        <v>867</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>864</v>
+        <v>868</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
@@ -7447,20 +7491,20 @@
         <v>151</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>865</v>
+        <v>869</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
+      <c r="I6" s="3"/>
     </row>
     <row r="7" ht="17" spans="1:9">
       <c r="A7" s="2" t="s">
-        <v>866</v>
+        <v>870</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>867</v>
+        <v>871</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>69</v>
@@ -7478,14 +7522,14 @@
         <v>487</v>
       </c>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="I7" s="3"/>
     </row>
     <row r="8" ht="17" spans="1:9">
       <c r="A8" s="2" t="s">
-        <v>868</v>
+        <v>872</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>869</v>
+        <v>873</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>80</v>
@@ -7494,7 +7538,7 @@
         <v>81</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>870</v>
+        <v>874</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>91</v>
@@ -7503,14 +7547,14 @@
         <v>487</v>
       </c>
       <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="I8" s="3"/>
     </row>
     <row r="9" ht="17" spans="1:9">
       <c r="A9" s="2" t="s">
-        <v>871</v>
+        <v>875</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>872</v>
+        <v>876</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>80</v>
@@ -7519,7 +7563,7 @@
         <v>81</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>873</v>
+        <v>877</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>439</v>
@@ -7528,23 +7572,23 @@
         <v>487</v>
       </c>
       <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="I9" s="3"/>
     </row>
     <row r="10" ht="17" spans="1:9">
       <c r="A10" s="2" t="s">
-        <v>874</v>
+        <v>878</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>876</v>
+        <v>880</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>877</v>
+        <v>881</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>173</v>
@@ -7553,14 +7597,14 @@
         <v>487</v>
       </c>
       <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="I10" s="3"/>
     </row>
     <row r="11" ht="17" spans="1:9">
       <c r="A11" s="2" t="s">
-        <v>878</v>
+        <v>882</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>879</v>
+        <v>883</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>80</v>
@@ -7569,77 +7613,77 @@
         <v>81</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>880</v>
+        <v>884</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>281</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="I11" s="3"/>
     </row>
     <row r="12" ht="17" spans="1:9">
       <c r="A12" s="2" t="s">
-        <v>881</v>
+        <v>885</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>882</v>
+        <v>886</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>883</v>
+        <v>887</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>884</v>
+        <v>888</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>885</v>
+        <v>889</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
+      <c r="I12" s="3"/>
     </row>
     <row r="13" ht="17" spans="1:9">
       <c r="A13" s="2" t="s">
-        <v>886</v>
+        <v>890</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>887</v>
+        <v>891</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>888</v>
+        <v>892</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>802</v>
+        <v>805</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>889</v>
+        <v>893</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
+      <c r="I13" s="3"/>
     </row>
     <row r="14" ht="17" spans="1:9">
       <c r="A14" s="2" t="s">
-        <v>890</v>
+        <v>894</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>891</v>
+        <v>895</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>574</v>
@@ -7651,7 +7695,7 @@
         <v>487</v>
       </c>
       <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+      <c r="I14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7703,82 +7747,82 @@
     </row>
     <row r="2" ht="17" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>893</v>
+        <v>897</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>894</v>
+        <v>898</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>850</v>
+        <v>853</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>895</v>
+        <v>899</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>896</v>
+        <v>900</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" ht="17" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>897</v>
+        <v>901</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>900</v>
+        <v>904</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>901</v>
+        <v>905</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" ht="34" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>902</v>
+        <v>906</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>903</v>
+        <v>907</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>904</v>
+        <v>908</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>905</v>
+        <v>909</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>906</v>
+        <v>910</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" ht="17" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>907</v>
+        <v>911</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>908</v>
+        <v>912</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>909</v>
+        <v>913</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>151</v>
@@ -7787,36 +7831,36 @@
         <v>152</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" ht="17" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>910</v>
+        <v>914</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>911</v>
+        <v>915</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>912</v>
+        <v>916</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>913</v>
+        <v>917</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>173</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" ht="17" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>914</v>
+        <v>918</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>915</v>
+        <v>919</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>80</v>
@@ -7825,20 +7869,20 @@
         <v>81</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>916</v>
+        <v>920</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>91</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="H7" s="3"/>
     </row>
     <row r="8" ht="17" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>917</v>
+        <v>921</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>918</v>
+        <v>922</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>80</v>
@@ -7847,26 +7891,26 @@
         <v>81</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>919</v>
+        <v>923</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>920</v>
+        <v>924</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="H8" s="3"/>
     </row>
     <row r="9" ht="17" spans="1:8">
       <c r="A9" s="2" t="s">
-        <v>921</v>
+        <v>925</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>922</v>
+        <v>926</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>923</v>
+        <v>927</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>151</v>
@@ -7875,51 +7919,51 @@
         <v>185</v>
       </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+      <c r="H9" s="3"/>
     </row>
     <row r="10" ht="17" spans="1:8">
       <c r="A10" s="2" t="s">
-        <v>924</v>
+        <v>928</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>925</v>
+        <v>929</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>926</v>
+        <v>930</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>927</v>
+        <v>931</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>928</v>
+        <v>932</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="H10" s="3"/>
     </row>
     <row r="11" ht="17" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>929</v>
+        <v>933</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>930</v>
+        <v>934</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>931</v>
+        <v>935</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>190</v>
       </c>
       <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+      <c r="H11" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7971,32 +8015,32 @@
     </row>
     <row r="2" ht="17" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>932</v>
+        <v>936</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>933</v>
+        <v>937</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>934</v>
+        <v>938</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>574</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>935</v>
+        <v>939</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" ht="17" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>936</v>
+        <v>940</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>937</v>
+        <v>941</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
@@ -8011,14 +8055,14 @@
         <v>161</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" ht="17" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>938</v>
+        <v>942</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>939</v>
+        <v>943</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
@@ -8033,14 +8077,14 @@
         <v>161</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" ht="17" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>940</v>
+        <v>944</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>941</v>
+        <v>945</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
@@ -8049,20 +8093,20 @@
         <v>81</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>942</v>
+        <v>946</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>943</v>
+        <v>947</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" ht="17" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>944</v>
+        <v>948</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>945</v>
+        <v>949</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
@@ -8071,42 +8115,42 @@
         <v>81</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>946</v>
+        <v>950</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" ht="17" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>948</v>
+        <v>952</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>949</v>
+        <v>953</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>574</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>950</v>
+        <v>954</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="H7" s="3"/>
     </row>
     <row r="8" ht="17" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>951</v>
+        <v>955</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>952</v>
+        <v>956</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>80</v>
@@ -8115,13 +8159,13 @@
         <v>81</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>954</v>
+        <v>958</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="H8" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8179,8 +8223,8 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="7"/>
+  <dimension ref="A1:I18"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -8189,9 +8233,10 @@
     <col min="5" max="5" width="34" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="27.34375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:8">
+    <row r="1" ht="22" customHeight="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>59</v>
       </c>
@@ -8217,12 +8262,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" ht="17" spans="1:8">
+    <row r="2" ht="17" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>955</v>
+        <v>959</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>956</v>
+        <v>960</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
@@ -8231,20 +8276,20 @@
         <v>81</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>957</v>
+        <v>961</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>134</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" ht="17" spans="1:8">
+      <c r="H2" s="3"/>
+    </row>
+    <row r="3" ht="17" spans="1:9">
       <c r="A3" s="2" t="s">
-        <v>958</v>
+        <v>962</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>959</v>
+        <v>963</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
@@ -8253,20 +8298,20 @@
         <v>81</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>960</v>
+        <v>964</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>961</v>
+        <v>965</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" ht="34" spans="1:8">
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" ht="34" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>962</v>
+        <v>966</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>963</v>
+        <v>967</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
@@ -8275,20 +8320,20 @@
         <v>81</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>964</v>
+        <v>968</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>134</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" ht="34" spans="1:8">
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" ht="34" spans="1:9">
       <c r="A5" s="2" t="s">
-        <v>965</v>
+        <v>969</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>966</v>
+        <v>970</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
@@ -8297,20 +8342,20 @@
         <v>81</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>967</v>
+        <v>971</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>968</v>
+        <v>972</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" ht="17" spans="1:8">
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" ht="17" spans="1:9">
       <c r="A6" s="2" t="s">
-        <v>969</v>
+        <v>973</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>970</v>
+        <v>974</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
@@ -8319,42 +8364,42 @@
         <v>81</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>971</v>
+        <v>975</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>134</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" ht="17" spans="1:8">
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" ht="17" spans="1:9">
       <c r="A7" s="2" t="s">
-        <v>972</v>
+        <v>976</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>973</v>
+        <v>977</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>974</v>
+        <v>978</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>975</v>
+        <v>979</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>976</v>
+        <v>980</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" ht="17" spans="1:8">
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" ht="17" spans="1:9">
       <c r="A8" s="2" t="s">
-        <v>977</v>
+        <v>981</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>978</v>
+        <v>982</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>69</v>
@@ -8363,20 +8408,23 @@
         <v>81</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>979</v>
+        <v>983</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>134</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" ht="17" spans="1:8">
+      <c r="H8" s="3"/>
+      <c r="I8" t="s">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="9" ht="17" spans="1:9">
       <c r="A9" s="2" t="s">
-        <v>980</v>
+        <v>985</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>981</v>
+        <v>986</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>80</v>
@@ -8385,20 +8433,20 @@
         <v>81</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>982</v>
+        <v>987</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>983</v>
+        <v>988</v>
       </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" ht="17" spans="1:8">
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" ht="17" spans="1:9">
       <c r="A10" s="2" t="s">
-        <v>984</v>
+        <v>989</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>985</v>
+        <v>990</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>80</v>
@@ -8407,20 +8455,20 @@
         <v>81</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>986</v>
+        <v>991</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>177</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" ht="17" spans="1:8">
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" ht="17" spans="1:9">
       <c r="A11" s="2" t="s">
-        <v>987</v>
+        <v>992</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>988</v>
+        <v>993</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>80</v>
@@ -8429,20 +8477,20 @@
         <v>81</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>989</v>
+        <v>994</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>990</v>
+        <v>995</v>
       </c>
       <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" ht="17" spans="1:8">
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" ht="17" spans="1:9">
       <c r="A12" s="2" t="s">
-        <v>991</v>
+        <v>996</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>992</v>
+        <v>997</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>80</v>
@@ -8451,20 +8499,20 @@
         <v>81</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>993</v>
+        <v>998</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>994</v>
+        <v>999</v>
       </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" ht="17" spans="1:8">
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" ht="17" spans="1:9">
       <c r="A13" s="2" t="s">
-        <v>995</v>
+        <v>1000</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>996</v>
+        <v>1001</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>80</v>
@@ -8473,20 +8521,20 @@
         <v>81</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>997</v>
+        <v>1002</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>439</v>
       </c>
       <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" ht="17" spans="1:8">
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" ht="17" spans="1:9">
       <c r="A14" s="2" t="s">
-        <v>998</v>
+        <v>1003</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>999</v>
+        <v>1004</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>80</v>
@@ -8495,20 +8543,20 @@
         <v>81</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>1000</v>
+        <v>1005</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>439</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" ht="17" spans="1:8">
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" ht="17" spans="1:9">
       <c r="A15" s="2" t="s">
-        <v>1001</v>
+        <v>1006</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>1002</v>
+        <v>1007</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>80</v>
@@ -8517,20 +8565,20 @@
         <v>81</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>1003</v>
+        <v>1008</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>181</v>
       </c>
       <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" ht="17" spans="1:8">
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" ht="17" spans="1:9">
       <c r="A16" s="2" t="s">
-        <v>1004</v>
+        <v>1009</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>1005</v>
+        <v>1010</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>80</v>
@@ -8539,20 +8587,20 @@
         <v>81</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>1006</v>
+        <v>1011</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>1007</v>
+        <v>1012</v>
       </c>
       <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
+      <c r="H16" s="3"/>
     </row>
     <row r="17" ht="17" spans="1:8">
       <c r="A17" s="2" t="s">
-        <v>1008</v>
+        <v>1013</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>1009</v>
+        <v>1014</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>80</v>
@@ -8561,35 +8609,35 @@
         <v>81</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>1010</v>
+        <v>1015</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>439</v>
       </c>
       <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
+      <c r="H17" s="3"/>
     </row>
     <row r="18" ht="17" spans="1:8">
       <c r="A18" s="2" t="s">
-        <v>1011</v>
+        <v>1016</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>1012</v>
+        <v>1017</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>1013</v>
+        <v>1018</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>1014</v>
+        <v>1019</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>1015</v>
+        <v>1020</v>
       </c>
       <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
+      <c r="H18" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8645,35 +8693,35 @@
     </row>
     <row r="2" ht="34" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>1016</v>
+        <v>1021</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1017</v>
+        <v>1022</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>850</v>
+        <v>853</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>1018</v>
+        <v>1023</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>1019</v>
+        <v>1024</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
+      <c r="I2" s="3"/>
     </row>
     <row r="3" ht="17" spans="1:9">
       <c r="A3" s="2" t="s">
-        <v>1020</v>
+        <v>1025</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1021</v>
+        <v>1026</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
@@ -8682,48 +8730,48 @@
         <v>81</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>1022</v>
+        <v>1027</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>1023</v>
+        <v>1028</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="I3" s="3"/>
     </row>
     <row r="4" ht="17" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>1024</v>
+        <v>1029</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1025</v>
+        <v>1030</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1026</v>
+        <v>1031</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>1027</v>
+        <v>1032</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>1028</v>
+        <v>1033</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
+      <c r="I4" s="3"/>
     </row>
     <row r="5" ht="17" spans="1:9">
       <c r="A5" s="2" t="s">
-        <v>1029</v>
+        <v>1034</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1030</v>
+        <v>1035</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
@@ -8732,46 +8780,46 @@
         <v>81</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1031</v>
+        <v>1036</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1032</v>
+        <v>1037</v>
       </c>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
+      <c r="I5" s="3"/>
     </row>
     <row r="6" ht="34" spans="1:9">
       <c r="A6" s="2" t="s">
-        <v>1033</v>
+        <v>1038</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1034</v>
+        <v>1039</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1035</v>
+        <v>1040</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1036</v>
+        <v>1041</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>1037</v>
+        <v>1042</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
+      <c r="I6" s="3"/>
     </row>
     <row r="7" ht="17" spans="1:9">
       <c r="A7" s="2" t="s">
-        <v>1038</v>
+        <v>1043</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1039</v>
+        <v>1044</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>69</v>
@@ -8780,21 +8828,21 @@
         <v>81</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1040</v>
+        <v>1045</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>1041</v>
+        <v>1046</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
+      <c r="I7" s="3"/>
     </row>
     <row r="8" ht="17" spans="1:9">
       <c r="A8" s="2" t="s">
-        <v>1042</v>
+        <v>1047</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1043</v>
+        <v>1048</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>80</v>
@@ -8803,7 +8851,7 @@
         <v>81</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>1044</v>
+        <v>1049</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>439</v>
@@ -8812,14 +8860,14 @@
         <v>487</v>
       </c>
       <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
+      <c r="I8" s="3"/>
     </row>
     <row r="9" ht="17" spans="1:9">
       <c r="A9" s="2" t="s">
-        <v>1045</v>
+        <v>1050</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>1046</v>
+        <v>1051</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>80</v>
@@ -8828,45 +8876,45 @@
         <v>81</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>1047</v>
+        <v>1052</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
+      <c r="I9" s="3"/>
     </row>
     <row r="10" ht="17" spans="1:9">
       <c r="A10" s="2" t="s">
-        <v>1049</v>
+        <v>1054</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1050</v>
+        <v>1055</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>1051</v>
+        <v>1056</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>1053</v>
+        <v>1058</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
+      <c r="I10" s="3"/>
     </row>
     <row r="11" ht="17" spans="1:9">
       <c r="A11" s="2" t="s">
-        <v>1054</v>
+        <v>1059</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>572</v>
@@ -8875,19 +8923,19 @@
         <v>80</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>892</v>
+        <v>896</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>1052</v>
+        <v>1057</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>1055</v>
+        <v>1060</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>487</v>
       </c>
       <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
+      <c r="I11" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8899,8 +8947,8 @@
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="7"/>
+  <dimension ref="A1:I14"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
@@ -8909,9 +8957,10 @@
     <col min="5" max="5" width="34" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="27.2109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:8">
+    <row r="1" ht="22" customHeight="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>59</v>
       </c>
@@ -8937,12 +8986,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" ht="17" spans="1:8">
+    <row r="2" ht="17" spans="1:9">
       <c r="A2" s="2" t="s">
-        <v>1056</v>
+        <v>1061</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1057</v>
+        <v>1062</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
@@ -8951,20 +9000,20 @@
         <v>112</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>1058</v>
+        <v>1063</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>134</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" ht="34" spans="1:8">
+      <c r="H2" s="3"/>
+    </row>
+    <row r="3" ht="34" spans="1:9">
       <c r="A3" s="2" t="s">
-        <v>1059</v>
+        <v>1064</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1060</v>
+        <v>1065</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
@@ -8973,20 +9022,20 @@
         <v>81</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>1061</v>
+        <v>1066</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>1062</v>
+        <v>1067</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" ht="34" spans="1:8">
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" ht="34" spans="1:9">
       <c r="A4" s="2" t="s">
-        <v>1063</v>
+        <v>1068</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1064</v>
+        <v>1069</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
@@ -8995,20 +9044,20 @@
         <v>81</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>1065</v>
+        <v>1070</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>1066</v>
+        <v>1071</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" ht="17" spans="1:8">
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" ht="17" spans="1:9">
       <c r="A5" s="2" t="s">
-        <v>1067</v>
+        <v>1072</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1068</v>
+        <v>1073</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
@@ -9017,86 +9066,89 @@
         <v>81</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1069</v>
+        <v>1074</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1070</v>
+        <v>1075</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" ht="17" spans="1:8">
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" ht="17" spans="1:9">
       <c r="A6" s="2" t="s">
-        <v>1071</v>
+        <v>1076</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1072</v>
+        <v>1077</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1073</v>
+        <v>1078</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1074</v>
+        <v>1079</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>1075</v>
+        <v>1080</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" ht="17" spans="1:8">
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" ht="17" spans="1:9">
       <c r="A7" s="2" t="s">
-        <v>1076</v>
+        <v>1081</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1077</v>
+        <v>1082</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1078</v>
+        <v>1083</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1079</v>
+        <v>1084</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>1080</v>
+        <v>1085</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" ht="17" spans="1:8">
+      <c r="H7" s="4"/>
+      <c r="I7" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="8" ht="17" spans="1:9">
       <c r="A8" s="2" t="s">
-        <v>1081</v>
+        <v>1087</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1082</v>
+        <v>1088</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1083</v>
+        <v>1089</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>1084</v>
+        <v>1090</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>1085</v>
+        <v>1091</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" ht="17" spans="1:8">
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" ht="17" spans="1:9">
       <c r="A9" s="2" t="s">
-        <v>1086</v>
+        <v>1092</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>1087</v>
+        <v>1093</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>80</v>
@@ -9105,42 +9157,42 @@
         <v>81</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>1088</v>
+        <v>1094</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>91</v>
       </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" ht="17" spans="1:8">
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" ht="17" spans="1:9">
       <c r="A10" s="2" t="s">
-        <v>1089</v>
+        <v>1095</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>875</v>
+        <v>879</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>1090</v>
+        <v>1096</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>1091</v>
+        <v>1097</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>173</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" ht="34" spans="1:8">
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" ht="34" spans="1:9">
       <c r="A11" s="2" t="s">
-        <v>1092</v>
+        <v>1098</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>1093</v>
+        <v>1099</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>80</v>
@@ -9149,20 +9201,20 @@
         <v>81</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>1094</v>
+        <v>1100</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>1048</v>
+        <v>1053</v>
       </c>
       <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" ht="17" spans="1:8">
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" ht="17" spans="1:9">
       <c r="A12" s="2" t="s">
-        <v>1095</v>
+        <v>1101</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1096</v>
+        <v>1102</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>80</v>
@@ -9171,20 +9223,20 @@
         <v>81</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>1097</v>
+        <v>1103</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>439</v>
       </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" ht="34" spans="1:8">
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" ht="34" spans="1:9">
       <c r="A13" s="2" t="s">
-        <v>1098</v>
+        <v>1104</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1099</v>
+        <v>1105</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>80</v>
@@ -9193,20 +9245,20 @@
         <v>81</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>1100</v>
+        <v>1106</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>1101</v>
+        <v>1107</v>
       </c>
       <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" ht="17" spans="1:8">
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" ht="17" spans="1:9">
       <c r="A14" s="2" t="s">
-        <v>1102</v>
+        <v>1108</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1103</v>
+        <v>1109</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>80</v>
@@ -9215,13 +9267,13 @@
         <v>81</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>1104</v>
+        <v>1110</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>439</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
+      <c r="H14" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9273,98 +9325,98 @@
     </row>
     <row r="2" ht="34" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>1105</v>
+        <v>1111</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1106</v>
+        <v>1112</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1107</v>
+        <v>1113</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>1108</v>
+        <v>1114</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>1109</v>
+        <v>1115</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" ht="17" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>1110</v>
+        <v>1116</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1111</v>
+        <v>1117</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1112</v>
+        <v>1118</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>1108</v>
+        <v>1114</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>1113</v>
+        <v>1119</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" ht="17" spans="1:8">
       <c r="A4" s="2" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>1122</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>1114</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>1115</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>1116</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>1108</v>
-      </c>
       <c r="F4" s="2" t="s">
-        <v>1117</v>
+        <v>1123</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" ht="17" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>1118</v>
+        <v>1124</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1119</v>
+        <v>1125</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1120</v>
+        <v>1126</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1108</v>
+        <v>1114</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1121</v>
+        <v>1127</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" ht="17" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>1122</v>
+        <v>1128</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1123</v>
+        <v>1129</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
@@ -9373,57 +9425,57 @@
         <v>81</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1108</v>
+        <v>1114</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>1124</v>
+        <v>1130</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" ht="17" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>1125</v>
+        <v>1131</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1126</v>
+        <v>1132</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1127</v>
+        <v>1133</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1108</v>
+        <v>1114</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>1128</v>
+        <v>1134</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="H7" s="3"/>
     </row>
     <row r="8" ht="17" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>1129</v>
+        <v>1135</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1130</v>
+        <v>1136</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>1131</v>
+        <v>1137</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>1108</v>
+        <v>1114</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>1132</v>
+        <v>1138</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="H8" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9475,120 +9527,120 @@
     </row>
     <row r="2" ht="17" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>1133</v>
+        <v>1139</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1134</v>
+        <v>1140</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>1135</v>
+        <v>1141</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>1136</v>
+        <v>1142</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>1137</v>
+        <v>1143</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" ht="17" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>1138</v>
+        <v>1144</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1139</v>
+        <v>1145</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1140</v>
+        <v>1146</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>1141</v>
+        <v>1147</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>1142</v>
+        <v>1148</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" ht="17" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>1143</v>
+        <v>1149</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1144</v>
+        <v>1150</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1145</v>
+        <v>1151</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>1146</v>
+        <v>1152</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>1147</v>
+        <v>1153</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" ht="17" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>1148</v>
+        <v>1154</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1149</v>
+        <v>1155</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1150</v>
+        <v>1156</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1151</v>
+        <v>1157</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1152</v>
+        <v>1158</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" ht="17" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>1153</v>
+        <v>1159</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1154</v>
+        <v>1160</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1155</v>
+        <v>1161</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1146</v>
+        <v>1152</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>1156</v>
+        <v>1162</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" ht="17" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>1157</v>
+        <v>1163</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1158</v>
+        <v>1164</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>80</v>
@@ -9597,13 +9649,13 @@
         <v>81</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1159</v>
+        <v>1165</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>1160</v>
+        <v>1166</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="H7" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9655,10 +9707,10 @@
     </row>
     <row r="2" ht="34" spans="1:8">
       <c r="A2" s="2" t="s">
-        <v>1161</v>
+        <v>1167</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>1162</v>
+        <v>1168</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>69</v>
@@ -9667,130 +9719,130 @@
         <v>81</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>1163</v>
+        <v>1169</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>1164</v>
+        <v>1170</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" ht="34" spans="1:8">
       <c r="A3" s="2" t="s">
-        <v>1165</v>
+        <v>1171</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1166</v>
+        <v>1172</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>1167</v>
+        <v>1173</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>1168</v>
+        <v>1174</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>1169</v>
+        <v>1175</v>
       </c>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="4" ht="34" spans="1:8">
       <c r="A4" s="2" t="s">
-        <v>1170</v>
+        <v>1176</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>1171</v>
+        <v>1177</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>1172</v>
+        <v>1178</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>1173</v>
+        <v>1179</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>1174</v>
+        <v>1180</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="H4" s="3"/>
     </row>
     <row r="5" ht="34" spans="1:8">
       <c r="A5" s="2" t="s">
-        <v>1175</v>
+        <v>1181</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>1176</v>
+        <v>1182</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>1172</v>
+        <v>1178</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>1177</v>
+        <v>1183</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>1178</v>
+        <v>1184</v>
       </c>
       <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="H5" s="3"/>
     </row>
     <row r="6" ht="51" spans="1:8">
       <c r="A6" s="2" t="s">
-        <v>1179</v>
+        <v>1185</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>1180</v>
+        <v>1186</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>1172</v>
+        <v>1178</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1181</v>
+        <v>1187</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>1182</v>
+        <v>1188</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="H6" s="3"/>
     </row>
     <row r="7" ht="34" spans="1:8">
       <c r="A7" s="2" t="s">
-        <v>1183</v>
+        <v>1189</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>1184</v>
+        <v>1190</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>1185</v>
+        <v>1191</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>1186</v>
+        <v>1192</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>1187</v>
+        <v>1193</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="H7" s="3"/>
     </row>
     <row r="8" ht="34" spans="1:8">
       <c r="A8" s="2" t="s">
-        <v>1188</v>
+        <v>1194</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>1189</v>
+        <v>1195</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>69</v>
@@ -9799,20 +9851,20 @@
         <v>81</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>1190</v>
+        <v>1196</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>1191</v>
+        <v>1197</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="H8" s="3"/>
     </row>
     <row r="9" ht="34" spans="1:8">
       <c r="A9" s="2" t="s">
-        <v>1192</v>
+        <v>1198</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>1193</v>
+        <v>1199</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>69</v>
@@ -9821,20 +9873,20 @@
         <v>588</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>1194</v>
+        <v>1200</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>1195</v>
+        <v>1201</v>
       </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+      <c r="H9" s="3"/>
     </row>
     <row r="10" ht="34" spans="1:8">
       <c r="A10" s="2" t="s">
-        <v>1196</v>
+        <v>1202</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>1197</v>
+        <v>1203</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>69</v>
@@ -9843,20 +9895,20 @@
         <v>81</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>1198</v>
+        <v>1204</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>1199</v>
+        <v>1205</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="H10" s="3"/>
     </row>
     <row r="11" ht="34" spans="1:8">
       <c r="A11" s="2" t="s">
-        <v>1200</v>
+        <v>1206</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>1201</v>
+        <v>1207</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>69</v>
@@ -9865,42 +9917,42 @@
         <v>81</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>1202</v>
+        <v>1208</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>1203</v>
+        <v>1209</v>
       </c>
       <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+      <c r="H11" s="3"/>
     </row>
     <row r="12" ht="34" spans="1:8">
       <c r="A12" s="2" t="s">
-        <v>1204</v>
+        <v>1210</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>1205</v>
+        <v>1211</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>69</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>1206</v>
+        <v>1212</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>1207</v>
+        <v>1213</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>1208</v>
+        <v>1214</v>
       </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
+      <c r="H12" s="3"/>
     </row>
     <row r="13" ht="34" spans="1:8">
       <c r="A13" s="2" t="s">
-        <v>1209</v>
+        <v>1215</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>1210</v>
+        <v>1216</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>80</v>
@@ -9909,42 +9961,42 @@
         <v>81</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>1211</v>
+        <v>1217</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>1212</v>
+        <v>1218</v>
       </c>
       <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
+      <c r="H13" s="3"/>
     </row>
     <row r="14" ht="34" spans="1:8">
       <c r="A14" s="2" t="s">
-        <v>1213</v>
+        <v>1219</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>1214</v>
+        <v>1220</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>80</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>1215</v>
+        <v>1221</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>1216</v>
+        <v>1222</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>1217</v>
+        <v>1223</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
+      <c r="H14" s="3"/>
     </row>
     <row r="15" ht="34" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>1218</v>
+        <v>1224</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>1219</v>
+        <v>1225</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>80</v>
@@ -9953,13 +10005,13 @@
         <v>81</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>1220</v>
+        <v>1226</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>1221</v>
+        <v>1227</v>
       </c>
       <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
+      <c r="H15" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9981,7 +10033,7 @@
     <col min="5" max="5" width="34" customWidth="1"/>
     <col min="6" max="6" width="48" customWidth="1"/>
     <col min="7" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="26.3046875" style="8" customWidth="1"/>
+    <col min="9" max="9" width="26.3046875" style="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:9">
@@ -10009,7 +10061,7 @@
       <c r="H1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="I1" s="10" t="s">
         <v>66</v>
       </c>
     </row>
@@ -10189,7 +10241,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="3"/>
     </row>
-    <row r="10" ht="17" spans="1:9">
+    <row r="10" ht="34" spans="1:9">
       <c r="A10" s="2" t="s">
         <v>104</v>
       </c>
@@ -10209,8 +10261,8 @@
         <v>108</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="10" t="s">
+      <c r="H10" s="5"/>
+      <c r="I10" s="12" t="s">
         <v>109</v>
       </c>
     </row>
@@ -10236,7 +10288,7 @@
       <c r="G11" s="2"/>
       <c r="H11" s="3"/>
     </row>
-    <row r="12" ht="17" spans="1:9">
+    <row r="12" ht="101" spans="1:9">
       <c r="A12" s="2" t="s">
         <v>115</v>
       </c>
@@ -10257,7 +10309,7 @@
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="3"/>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="12" t="s">
         <v>120</v>
       </c>
     </row>
@@ -10865,8 +10917,8 @@
         <v>223</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="11" t="s">
+      <c r="H8" s="7"/>
+      <c r="I8" s="13" t="s">
         <v>224</v>
       </c>
     </row>
@@ -10905,7 +10957,7 @@
       <c r="D10" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="6" t="s">
         <v>232</v>
       </c>
       <c r="F10" s="2" t="s">
@@ -11045,7 +11097,7 @@
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="3"/>
-      <c r="I16" s="11" t="s">
+      <c r="I16" s="13" t="s">
         <v>260</v>
       </c>
     </row>
@@ -11114,7 +11166,7 @@
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="3"/>
-      <c r="I19" s="11" t="s">
+      <c r="I19" s="13" t="s">
         <v>274</v>
       </c>
     </row>
@@ -11314,8 +11366,8 @@
         <v>307</v>
       </c>
       <c r="G28" s="2"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="12" t="s">
+      <c r="H28" s="5"/>
+      <c r="I28" s="14" t="s">
         <v>308</v>
       </c>
     </row>
@@ -11339,8 +11391,8 @@
         <v>312</v>
       </c>
       <c r="G29" s="2"/>
-      <c r="H29" s="6"/>
-      <c r="I29" s="12" t="s">
+      <c r="H29" s="5"/>
+      <c r="I29" s="14" t="s">
         <v>313</v>
       </c>
     </row>

</xml_diff>